<commit_message>
more bikes and filters
</commit_message>
<xml_diff>
--- a/data/gravel incomplete/BlackMtnCy La Cabra 2022.xlsx
+++ b/data/gravel incomplete/BlackMtnCy La Cabra 2022.xlsx
@@ -1,265 +1,290 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/walker/Documents/Github/Bike Geometry Project/data/gravel incomplete/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EE3D7A-5B79-7743-A4B6-837FF3282E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="13120" windowHeight="6100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
-  <si>
-    <t xml:space="preserve">brand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BlackMtnCy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">model</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="86">
+  <si>
+    <t>brand</t>
+  </si>
+  <si>
+    <t>BlackMtnCy</t>
+  </si>
+  <si>
+    <t>model</t>
   </si>
   <si>
     <t xml:space="preserve">La Cabra </t>
   </si>
   <si>
-    <t xml:space="preserve">model_year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">url</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a8:g32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frame_size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frame size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seat_tube_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">head_tube_angle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seat_tube_angle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">top_tube_effective_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chainstay_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bottom_bracket_drop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">head_tube_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">axle_crown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fork_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fork_offset_rake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">standover</t>
-  </si>
-  <si>
-    <t xml:space="preserve">front_center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wheelbase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crank_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">handlebar_width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stem_length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frame_weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wheel_size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tire_width_spec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tire_width_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rider_min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rider_max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spec_list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">steel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dropout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tire_width_max_700c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tire_width_max_650b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">suspension_corrected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fork_suspension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stem_suspension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rear_suspension</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rear_axle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">front_axle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bottom_bracket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q_factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seatpost_diameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">front_derailleur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_chainring_1x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_chainring_2x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rotor_max_front</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rotor_max_rear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iso_astm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">routing_shifter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">routing_dropper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">routing_dynamo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">internal_storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_inner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_under</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_top</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_fork</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_fender</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_rack_front</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mounts_rack_rear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frameset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">base_build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">custom_builds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">currency</t>
+    <t>model_year</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>input_date</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>data_range</t>
+  </si>
+  <si>
+    <t>a8:g32</t>
+  </si>
+  <si>
+    <t>frame_size</t>
+  </si>
+  <si>
+    <t>frame size</t>
+  </si>
+  <si>
+    <t>15"</t>
+  </si>
+  <si>
+    <t>16"</t>
+  </si>
+  <si>
+    <t>18"</t>
+  </si>
+  <si>
+    <t>20"</t>
+  </si>
+  <si>
+    <t>22"</t>
+  </si>
+  <si>
+    <t>seat_tube_length</t>
+  </si>
+  <si>
+    <t>head_tube_angle</t>
+  </si>
+  <si>
+    <t>seat_tube_angle</t>
+  </si>
+  <si>
+    <t>top_tube_effective_length</t>
+  </si>
+  <si>
+    <t>chainstay_length</t>
+  </si>
+  <si>
+    <t>bottom_bracket_drop</t>
+  </si>
+  <si>
+    <t>head_tube_length</t>
+  </si>
+  <si>
+    <t>axle_crown</t>
+  </si>
+  <si>
+    <t>fork_length</t>
+  </si>
+  <si>
+    <t>fork_offset_rake</t>
+  </si>
+  <si>
+    <t>trail</t>
+  </si>
+  <si>
+    <t>stack</t>
+  </si>
+  <si>
+    <t>reach</t>
+  </si>
+  <si>
+    <t>standover</t>
+  </si>
+  <si>
+    <t>front_center</t>
+  </si>
+  <si>
+    <t>wheelbase</t>
+  </si>
+  <si>
+    <t>crank_length</t>
+  </si>
+  <si>
+    <t>handlebar_width</t>
+  </si>
+  <si>
+    <t>stem_length</t>
+  </si>
+  <si>
+    <t>frame_weight</t>
+  </si>
+  <si>
+    <t>wheel_size</t>
+  </si>
+  <si>
+    <t>tire_width_spec</t>
+  </si>
+  <si>
+    <t>tire_width_max</t>
+  </si>
+  <si>
+    <t>rider_min</t>
+  </si>
+  <si>
+    <t>rider_max</t>
+  </si>
+  <si>
+    <t>spec_list</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>material</t>
+  </si>
+  <si>
+    <t>steel</t>
+  </si>
+  <si>
+    <t>udh</t>
+  </si>
+  <si>
+    <t>dropout</t>
+  </si>
+  <si>
+    <t>tire_width_max_700c</t>
+  </si>
+  <si>
+    <t>tire_width_max_650b</t>
+  </si>
+  <si>
+    <t>suspension_corrected</t>
+  </si>
+  <si>
+    <t>fork_suspension</t>
+  </si>
+  <si>
+    <t>stem_suspension</t>
+  </si>
+  <si>
+    <t>rear_suspension</t>
+  </si>
+  <si>
+    <t>rear_axle</t>
+  </si>
+  <si>
+    <t>front_axle</t>
+  </si>
+  <si>
+    <t>bottom_bracket</t>
+  </si>
+  <si>
+    <t>q_factor</t>
+  </si>
+  <si>
+    <t>seatpost_diameter</t>
+  </si>
+  <si>
+    <t>front_derailleur</t>
+  </si>
+  <si>
+    <t>max_chainring_1x</t>
+  </si>
+  <si>
+    <t>max_chainring_2x</t>
+  </si>
+  <si>
+    <t>rotor_max_front</t>
+  </si>
+  <si>
+    <t>rotor_max_rear</t>
+  </si>
+  <si>
+    <t>iso_astm</t>
+  </si>
+  <si>
+    <t>routing_shifter</t>
+  </si>
+  <si>
+    <t>routing_dropper</t>
+  </si>
+  <si>
+    <t>routing_dynamo</t>
+  </si>
+  <si>
+    <t>internal_storage</t>
+  </si>
+  <si>
+    <t>mounts_inner</t>
+  </si>
+  <si>
+    <t>mounts_under</t>
+  </si>
+  <si>
+    <t>mounts_top</t>
+  </si>
+  <si>
+    <t>mounts_fork</t>
+  </si>
+  <si>
+    <t>mounts_fender</t>
+  </si>
+  <si>
+    <t>mounts_rack_front</t>
+  </si>
+  <si>
+    <t>mounts_rack_rear</t>
+  </si>
+  <si>
+    <t>frameset</t>
+  </si>
+  <si>
+    <t>base_build</t>
+  </si>
+  <si>
+    <t>custom_builds</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>class</t>
+  </si>
+  <si>
+    <t>gravel</t>
+  </si>
+  <si>
+    <t>handlebar</t>
+  </si>
+  <si>
+    <t>drop bar</t>
+  </si>
+  <si>
+    <t>fork</t>
+  </si>
+  <si>
+    <t>rigid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
@@ -293,6 +318,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -574,15 +608,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="19.71" hidden="0" customWidth="1"/>
+    <col min="1" max="2" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -590,7 +623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -598,7 +631,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -606,7 +639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -614,13 +647,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5"/>
-    </row>
-    <row r="7">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -628,7 +660,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -651,513 +683,490 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>380</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>405</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>460</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>508</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>560</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>70</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>70</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>70.5</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>70.5</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>70.5</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>74</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>73.5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>73</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>72.5</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>72.5</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>545</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>560</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>580</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>600</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>620</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>444</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>444</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>444</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>444</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>444</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>22</v>
       </c>
       <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>70</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>70</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>70</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>70</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>125</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>150</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>175</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>205</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>230</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>24</v>
       </c>
       <c r="B16" t="s">
         <v>25</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>425</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>425</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>425</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>425</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>425</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
       <c r="B17" t="s">
         <v>26</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>55</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>55</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>50</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>50</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>50</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18">
         <v>72</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18">
         <v>72</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18">
         <v>74</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18">
         <v>74</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18">
         <v>74</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
       <c r="B19" t="s">
         <v>28</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19">
         <v>581</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19">
         <v>604</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19">
         <v>632</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19">
         <v>660</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19">
         <v>684</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
       <c r="B20" t="s">
         <v>29</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20">
         <v>376</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20">
         <v>378</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20">
         <v>385</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20">
         <v>390</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20">
         <v>403</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
       <c r="B21" t="s">
         <v>30</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21">
         <v>736</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21">
         <v>760</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21">
         <v>799</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21">
         <v>836</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21">
         <v>872</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
       <c r="B22" t="s">
         <v>31</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22">
         <v>624</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22">
         <v>635</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22">
         <v>641</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22">
         <v>656</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22">
         <v>677</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
       <c r="B23" t="s">
         <v>32</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23">
         <v>1059</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23">
         <v>1070</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23">
         <v>1075</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23">
         <v>1091</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23">
         <v>1112</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
       </c>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-    </row>
-    <row r="25">
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
       <c r="B25" t="s">
         <v>34</v>
       </c>
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-    </row>
-    <row r="26">
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
       <c r="B26" t="s">
         <v>35</v>
       </c>
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-    </row>
-    <row r="27">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-    </row>
-    <row r="28">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
       <c r="B28" t="s">
         <v>37</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28">
         <v>29</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28">
         <v>30</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E28">
         <v>31</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28">
         <v>32</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28">
         <v>33</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29">
         <v>60.96</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29">
         <v>60.96</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29">
         <v>60.96</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29">
         <v>60.96</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G29">
         <v>60.96</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30">
         <v>71.12</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D30">
         <v>71.12</v>
       </c>
-      <c r="E30" t="n">
+      <c r="E30">
         <v>71.12</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F30">
         <v>71.12</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G30">
         <v>71.12</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
-      <c r="B31"/>
-      <c r="C31" t="n">
+      <c r="C31">
         <v>152.4</v>
       </c>
-      <c r="D31" t="n">
-        <v>163.83</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D31">
+        <v>163.83000000000001</v>
+      </c>
+      <c r="E31">
         <v>171.45</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31">
         <v>179.07</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31">
         <v>186.69</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>41</v>
       </c>
-      <c r="B32"/>
-      <c r="C32" t="n">
-        <v>163.83</v>
-      </c>
-      <c r="D32" t="n">
+      <c r="C32">
+        <v>163.83000000000001</v>
+      </c>
+      <c r="D32">
         <v>171.45</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E32">
         <v>179.07</v>
       </c>
-      <c r="F32" t="n">
+      <c r="F32">
         <v>186.69</v>
       </c>
-      <c r="G32" t="n">
+      <c r="G32">
         <v>198.12</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1165,220 +1174,210 @@
         <v>43</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>44</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B38" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>46</v>
       </c>
-      <c r="B36"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>47</v>
       </c>
-      <c r="B37"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>48</v>
       </c>
-      <c r="B38"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>49</v>
       </c>
-      <c r="B39"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="s">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>50</v>
       </c>
-      <c r="B40"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="s">
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>51</v>
       </c>
-      <c r="B41"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>52</v>
       </c>
-      <c r="B42"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="s">
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
         <v>53</v>
       </c>
-      <c r="B43"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="s">
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>54</v>
       </c>
-      <c r="B44"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="s">
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>55</v>
       </c>
-      <c r="B45"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="s">
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>56</v>
       </c>
-      <c r="B46"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="s">
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
         <v>57</v>
       </c>
-      <c r="B47"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="s">
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>58</v>
       </c>
-      <c r="B48"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="s">
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>59</v>
       </c>
-      <c r="B49"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="s">
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>60</v>
       </c>
-      <c r="B50"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="s">
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>61</v>
       </c>
-      <c r="B51"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="s">
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>62</v>
       </c>
-      <c r="B52"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="s">
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>63</v>
       </c>
-      <c r="B53"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="s">
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>64</v>
       </c>
-      <c r="B54"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="s">
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
         <v>65</v>
       </c>
-      <c r="B55"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="s">
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>66</v>
       </c>
-      <c r="B56"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="s">
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>67</v>
       </c>
-      <c r="B57"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="s">
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>68</v>
       </c>
-      <c r="B58"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="s">
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>69</v>
       </c>
-      <c r="B59"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="s">
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>70</v>
       </c>
-      <c r="B60"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="s">
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>71</v>
       </c>
-      <c r="B61"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="s">
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>72</v>
       </c>
-      <c r="B62"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="s">
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
         <v>73</v>
       </c>
-      <c r="B63"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="s">
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
         <v>74</v>
       </c>
-      <c r="B64"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="s">
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
         <v>75</v>
       </c>
-      <c r="B65"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="s">
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>76</v>
       </c>
-      <c r="B66"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="s">
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>77</v>
       </c>
-      <c r="B67"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="s">
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
         <v>78</v>
       </c>
-      <c r="B68"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="s">
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
         <v>79</v>
       </c>
-      <c r="B69"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>